<commit_message>
auto commit 2026-05-11 21:56:10
</commit_message>
<xml_diff>
--- a/results_BK_SM.xlsx
+++ b/results_BK_SM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/akahmad/Documents/G-ThinkerCG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69EACB54-A5FF-2D47-B209-BDE2AE9F6BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A26C16B-92FC-A947-9E35-2C158E3C4CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="6" xr2:uid="{93E1CCD5-64A0-5F4C-A5F1-EE4B217F183B}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6594" uniqueCount="3986">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6611" uniqueCount="3988">
   <si>
     <t>amazon0601</t>
   </si>
@@ -11991,19 +11991,25 @@
     <t>Top Level Tasks</t>
   </si>
   <si>
-    <t xml:space="preserve">Flixster </t>
-  </si>
-  <si>
-    <t>OOT: 30m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Non-maximal removing </t>
-  </si>
-  <si>
     <t>Parallel</t>
   </si>
   <si>
     <t>Serial</t>
+  </si>
+  <si>
+    <t>min_size</t>
+  </si>
+  <si>
+    <t>gamma</t>
+  </si>
+  <si>
+    <t>Flixter</t>
+  </si>
+  <si>
+    <t>top level tasks</t>
+  </si>
+  <si>
+    <t>Time</t>
   </si>
 </sst>
 </file>
@@ -12015,7 +12021,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="34" x14ac:knownFonts="1">
+  <fonts count="40" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -12186,6 +12192,13 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="16"/>
       <color theme="1"/>
@@ -12221,6 +12234,36 @@
     <font>
       <b/>
       <sz val="14"/>
+      <name val="Monaco"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <name val="Monaco"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Monaco"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Monaco"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Display"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="18"/>
       <name val="Monaco"/>
       <family val="2"/>
     </font>
@@ -12361,7 +12404,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -12484,29 +12527,40 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -40565,9 +40619,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ED88F32-C306-9942-B2BF-61C867C9C8AC}">
-  <dimension ref="B3:AJ18"/>
+  <dimension ref="B4:AJ27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="59.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -40576,8 +40631,8 @@
     <col min="7" max="7" width="14.1640625" customWidth="1"/>
     <col min="8" max="8" width="15.5" customWidth="1"/>
     <col min="9" max="10" width="16.6640625" customWidth="1"/>
-    <col min="11" max="11" width="7.83203125" customWidth="1"/>
-    <col min="12" max="12" width="8.1640625" customWidth="1"/>
+    <col min="11" max="11" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
     <col min="14" max="14" width="9.6640625" customWidth="1"/>
     <col min="15" max="16" width="14.5" bestFit="1" customWidth="1"/>
@@ -40585,55 +40640,98 @@
     <col min="18" max="18" width="3.83203125" customWidth="1"/>
     <col min="19" max="19" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:36" x14ac:dyDescent="0.2">
-      <c r="AE3" t="s">
-        <v>3981</v>
-      </c>
-      <c r="AF3">
-        <v>23</v>
-      </c>
-      <c r="AG3">
+    <row r="4" spans="2:36" ht="19" x14ac:dyDescent="0.25">
+      <c r="W4" s="102" t="s">
+        <v>3972</v>
+      </c>
+      <c r="X4" s="102" t="s">
+        <v>3985</v>
+      </c>
+      <c r="AA4" s="103" t="s">
+        <v>3942</v>
+      </c>
+      <c r="AB4" s="105" t="s">
+        <v>3987</v>
+      </c>
+      <c r="AD4" s="103" t="s">
+        <v>3938</v>
+      </c>
+      <c r="AE4" s="105" t="s">
+        <v>3987</v>
+      </c>
+    </row>
+    <row r="5" spans="2:36" ht="26" x14ac:dyDescent="0.35">
+      <c r="W5" s="102" t="s">
+        <v>3983</v>
+      </c>
+      <c r="X5" s="102">
+        <v>30</v>
+      </c>
+      <c r="AA5" s="104">
+        <v>100</v>
+      </c>
+      <c r="AB5" s="107">
+        <v>111.26600000000001</v>
+      </c>
+      <c r="AD5" s="104">
+        <v>1</v>
+      </c>
+      <c r="AE5" s="106">
+        <v>19.003499999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="2:36" ht="26" x14ac:dyDescent="0.35">
+      <c r="W6" s="102" t="s">
+        <v>3984</v>
+      </c>
+      <c r="X6" s="102">
         <v>0.95</v>
       </c>
-    </row>
-    <row r="5" spans="2:36" x14ac:dyDescent="0.2">
-      <c r="AI5" t="s">
-        <v>3938</v>
-      </c>
-    </row>
-    <row r="6" spans="2:36" ht="22" x14ac:dyDescent="0.25">
-      <c r="AE6" s="91">
-        <v>0.7</v>
-      </c>
-      <c r="AF6" s="90">
-        <v>37.5715</v>
-      </c>
-      <c r="AI6">
-        <v>50</v>
-      </c>
-      <c r="AJ6" s="35">
-        <v>29.476199999999999</v>
-      </c>
+      <c r="AA6" s="104">
+        <v>1000</v>
+      </c>
+      <c r="AB6" s="107">
+        <v>29.1617</v>
+      </c>
+      <c r="AD6" s="104">
+        <v>10</v>
+      </c>
+      <c r="AE6" s="106">
+        <v>18.909700000000001</v>
+      </c>
+      <c r="AF6" s="90"/>
+      <c r="AJ6" s="35"/>
     </row>
     <row r="7" spans="2:36" ht="27" x14ac:dyDescent="0.35">
-      <c r="O7" s="97" t="s">
-        <v>3984</v>
-      </c>
+      <c r="O7" s="97"/>
       <c r="P7" s="97"/>
       <c r="Q7" s="97"/>
       <c r="R7" s="96"/>
-      <c r="S7" s="95" t="s">
-        <v>3985</v>
-      </c>
+      <c r="S7" s="95"/>
       <c r="T7" s="95"/>
-      <c r="AE7" s="91">
-        <v>0.8</v>
-      </c>
-      <c r="AF7" s="90">
-        <v>29.638500000000001</v>
-      </c>
+      <c r="W7" s="102" t="s">
+        <v>3986</v>
+      </c>
+      <c r="X7" s="92">
+        <v>36085</v>
+      </c>
+      <c r="AA7" s="104">
+        <v>10000</v>
+      </c>
+      <c r="AB7" s="107">
+        <v>18.9161</v>
+      </c>
+      <c r="AD7" s="104">
+        <v>20</v>
+      </c>
+      <c r="AE7" s="106">
+        <v>17.566099999999999</v>
+      </c>
+      <c r="AF7" s="90"/>
     </row>
     <row r="8" spans="2:36" ht="27" x14ac:dyDescent="0.35">
       <c r="B8" s="85" t="s">
@@ -40652,43 +40750,29 @@
       <c r="G8" s="85" t="s">
         <v>3971</v>
       </c>
-      <c r="J8" s="85" t="s">
-        <v>3972</v>
-      </c>
-      <c r="K8" s="85" t="s">
-        <v>3962</v>
-      </c>
-      <c r="L8" s="85" t="s">
-        <v>3963</v>
-      </c>
-      <c r="M8" s="85" t="s">
-        <v>3980</v>
-      </c>
-      <c r="O8" s="85" t="s">
-        <v>3929</v>
-      </c>
-      <c r="P8" s="85" t="s">
-        <v>3948</v>
-      </c>
-      <c r="Q8" s="85" t="s">
-        <v>3949</v>
-      </c>
+      <c r="J8" s="85"/>
+      <c r="K8" s="85"/>
+      <c r="L8" s="85"/>
+      <c r="M8" s="85"/>
+      <c r="O8" s="85"/>
+      <c r="P8" s="85"/>
+      <c r="Q8" s="85"/>
       <c r="R8" s="85"/>
-      <c r="S8" s="85" t="s">
-        <v>3934</v>
-      </c>
-      <c r="T8" s="85" t="s">
-        <v>3971</v>
-      </c>
-      <c r="W8" s="85" t="s">
-        <v>3983</v>
-      </c>
-      <c r="AE8" s="91">
-        <v>0.9</v>
-      </c>
-      <c r="AF8" s="90">
-        <v>30.749099999999999</v>
-      </c>
+      <c r="S8" s="85"/>
+      <c r="T8" s="85"/>
+      <c r="AA8" s="104">
+        <v>20000</v>
+      </c>
+      <c r="AB8" s="107">
+        <v>28.322800000000001</v>
+      </c>
+      <c r="AD8" s="104">
+        <v>50</v>
+      </c>
+      <c r="AE8" s="106">
+        <v>20.896999999999998</v>
+      </c>
+      <c r="AF8" s="90"/>
     </row>
     <row r="9" spans="2:36" ht="27" x14ac:dyDescent="0.35">
       <c r="B9" s="83" t="s">
@@ -40707,44 +40791,19 @@
       <c r="G9" s="87">
         <v>0.01</v>
       </c>
-      <c r="J9" s="85" t="s">
-        <v>1531</v>
-      </c>
-      <c r="K9" s="92">
-        <v>32</v>
-      </c>
-      <c r="L9" s="92">
-        <v>0.95</v>
-      </c>
-      <c r="M9" s="92">
-        <v>36085</v>
-      </c>
+      <c r="J9" s="85"/>
+      <c r="K9" s="92"/>
+      <c r="L9" s="92"/>
+      <c r="M9" s="92"/>
       <c r="N9" s="92"/>
-      <c r="O9" s="93">
-        <v>592.03700000000003</v>
-      </c>
-      <c r="P9" s="93">
-        <v>98.700100000000006</v>
-      </c>
-      <c r="Q9" s="98">
-        <v>28.236799999999999</v>
-      </c>
+      <c r="O9" s="93"/>
+      <c r="P9" s="93"/>
+      <c r="Q9" s="98"/>
       <c r="R9" s="93"/>
-      <c r="S9" s="93" t="s">
-        <v>3902</v>
-      </c>
-      <c r="T9" s="93">
-        <v>396.8</v>
-      </c>
-      <c r="W9">
-        <v>0.65</v>
-      </c>
-      <c r="AE9" s="91">
-        <v>0.95</v>
-      </c>
-      <c r="AF9" s="90">
-        <v>32.062800000000003</v>
-      </c>
+      <c r="S9" s="93"/>
+      <c r="T9" s="93"/>
+      <c r="AE9" s="91"/>
+      <c r="AF9" s="90"/>
     </row>
     <row r="10" spans="2:36" ht="27" x14ac:dyDescent="0.35">
       <c r="B10" s="83" t="s">
@@ -40763,41 +40822,19 @@
       <c r="G10" s="87">
         <v>0.22</v>
       </c>
-      <c r="J10" s="85" t="s">
-        <v>3979</v>
-      </c>
-      <c r="K10" s="92">
-        <v>23</v>
-      </c>
-      <c r="L10" s="92">
-        <v>0.9</v>
-      </c>
-      <c r="M10" s="92">
-        <v>16009</v>
-      </c>
+      <c r="J10" s="85"/>
+      <c r="K10" s="92"/>
+      <c r="L10" s="92"/>
+      <c r="M10" s="92"/>
       <c r="N10" s="92"/>
-      <c r="O10" s="93" t="s">
-        <v>3902</v>
-      </c>
-      <c r="P10" s="93">
-        <v>366.37599999999998</v>
-      </c>
-      <c r="Q10" s="98">
-        <v>267.767</v>
-      </c>
+      <c r="O10" s="93"/>
+      <c r="P10" s="93"/>
+      <c r="Q10" s="98"/>
       <c r="R10" s="93"/>
-      <c r="S10" s="93" t="s">
-        <v>3902</v>
-      </c>
-      <c r="T10" s="93" t="s">
-        <v>3902</v>
-      </c>
-      <c r="AE10" s="91">
-        <v>1</v>
-      </c>
-      <c r="AF10" s="91">
-        <v>101.65</v>
-      </c>
+      <c r="S10" s="93"/>
+      <c r="T10" s="93"/>
+      <c r="AE10" s="91"/>
+      <c r="AF10" s="91"/>
     </row>
     <row r="11" spans="2:36" ht="27" x14ac:dyDescent="0.35">
       <c r="B11" s="83" t="s">
@@ -40816,34 +40853,34 @@
       <c r="G11" s="87">
         <v>49.23</v>
       </c>
-      <c r="J11" s="85" t="s">
-        <v>1514</v>
-      </c>
-      <c r="K11" s="92">
-        <v>5</v>
-      </c>
-      <c r="L11" s="92">
-        <v>0.8</v>
-      </c>
-      <c r="M11" s="92">
-        <v>94500</v>
-      </c>
+      <c r="J11" s="85"/>
+      <c r="K11" s="92"/>
+      <c r="L11" s="92"/>
+      <c r="M11" s="92"/>
       <c r="N11" s="92"/>
-      <c r="O11" s="93">
-        <v>50.255800000000001</v>
-      </c>
-      <c r="P11" s="93">
-        <v>50.8005</v>
-      </c>
-      <c r="Q11" s="98">
-        <v>8.9690399999999997</v>
-      </c>
+      <c r="O11" s="93"/>
+      <c r="P11" s="93"/>
+      <c r="Q11" s="98"/>
       <c r="R11" s="93"/>
-      <c r="S11" s="93">
-        <v>235.078</v>
-      </c>
-      <c r="T11" s="93">
-        <v>296.74</v>
+      <c r="S11" s="93"/>
+      <c r="T11" s="93"/>
+      <c r="W11" s="102" t="s">
+        <v>3972</v>
+      </c>
+      <c r="X11" s="102" t="s">
+        <v>1528</v>
+      </c>
+      <c r="AA11" s="103" t="s">
+        <v>3942</v>
+      </c>
+      <c r="AB11" s="105" t="s">
+        <v>3987</v>
+      </c>
+      <c r="AD11" s="103" t="s">
+        <v>3938</v>
+      </c>
+      <c r="AE11" s="105" t="s">
+        <v>3987</v>
       </c>
     </row>
     <row r="12" spans="2:36" ht="27" x14ac:dyDescent="0.35">
@@ -40863,34 +40900,34 @@
       <c r="G12" s="87">
         <v>0.49</v>
       </c>
-      <c r="J12" s="85" t="s">
-        <v>1528</v>
-      </c>
-      <c r="K12" s="92">
-        <v>23</v>
-      </c>
-      <c r="L12" s="92">
-        <v>0.9</v>
-      </c>
-      <c r="M12" s="92">
-        <v>2517</v>
-      </c>
+      <c r="J12" s="85"/>
+      <c r="K12" s="92"/>
+      <c r="L12" s="92"/>
+      <c r="M12" s="92"/>
       <c r="N12" s="92"/>
-      <c r="O12" s="93">
-        <v>3.0164800000000001</v>
-      </c>
-      <c r="P12" s="93">
-        <v>4.6988599999999998</v>
-      </c>
-      <c r="Q12" s="93">
-        <v>1.30826</v>
-      </c>
+      <c r="O12" s="93"/>
+      <c r="P12" s="93"/>
+      <c r="Q12" s="93"/>
       <c r="R12" s="93"/>
-      <c r="S12" s="93">
-        <v>55.46</v>
-      </c>
-      <c r="T12" s="98">
-        <v>0.5</v>
+      <c r="S12" s="93"/>
+      <c r="T12" s="98"/>
+      <c r="W12" s="102" t="s">
+        <v>3983</v>
+      </c>
+      <c r="X12" s="102">
+        <v>20</v>
+      </c>
+      <c r="AA12">
+        <v>10</v>
+      </c>
+      <c r="AB12" s="82">
+        <v>112.94799999999999</v>
+      </c>
+      <c r="AD12" s="104">
+        <v>1</v>
+      </c>
+      <c r="AE12" s="82">
+        <v>23.771899999999999</v>
       </c>
     </row>
     <row r="13" spans="2:36" ht="23" x14ac:dyDescent="0.3">
@@ -40910,6 +40947,24 @@
       <c r="G13" s="87">
         <v>3.05</v>
       </c>
+      <c r="W13" s="102" t="s">
+        <v>3984</v>
+      </c>
+      <c r="X13" s="102">
+        <v>0.8</v>
+      </c>
+      <c r="AA13" s="104">
+        <v>100</v>
+      </c>
+      <c r="AB13" s="82">
+        <v>34.610700000000001</v>
+      </c>
+      <c r="AD13" s="104">
+        <v>10</v>
+      </c>
+      <c r="AE13" s="82">
+        <v>23.1478</v>
+      </c>
     </row>
     <row r="14" spans="2:36" ht="23" x14ac:dyDescent="0.3">
       <c r="B14" s="83" t="s">
@@ -40928,20 +40983,235 @@
       <c r="G14" s="87">
         <v>0.47</v>
       </c>
-      <c r="Q14" s="94" t="s">
-        <v>3982</v>
-      </c>
+      <c r="Q14" s="94"/>
       <c r="R14" s="94"/>
-    </row>
-    <row r="18" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="W14" s="102" t="s">
+        <v>3986</v>
+      </c>
+      <c r="X14" s="92">
+        <v>3785</v>
+      </c>
+      <c r="AA14" s="104">
+        <v>1000</v>
+      </c>
+      <c r="AB14" s="82">
+        <v>24.2639</v>
+      </c>
+      <c r="AD14" s="104">
+        <v>20</v>
+      </c>
+      <c r="AE14" s="82">
+        <v>23.116099999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="2:36" ht="22" x14ac:dyDescent="0.25">
+      <c r="AA15" s="104">
+        <v>10000</v>
+      </c>
+      <c r="AB15" s="82">
+        <v>30.773599999999998</v>
+      </c>
+      <c r="AD15" s="104">
+        <v>50</v>
+      </c>
+      <c r="AE15" s="82">
+        <v>24.661000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
       <c r="F18" t="s">
         <v>3974</v>
       </c>
     </row>
+    <row r="20" spans="2:14" ht="27" x14ac:dyDescent="0.35">
+      <c r="G20" s="97" t="s">
+        <v>3981</v>
+      </c>
+      <c r="H20" s="97"/>
+      <c r="I20" s="97"/>
+      <c r="J20" s="96"/>
+      <c r="K20" s="95" t="s">
+        <v>3982</v>
+      </c>
+      <c r="L20" s="95"/>
+    </row>
+    <row r="21" spans="2:14" ht="27" x14ac:dyDescent="0.35">
+      <c r="B21" s="85" t="s">
+        <v>3972</v>
+      </c>
+      <c r="C21" s="85" t="s">
+        <v>3983</v>
+      </c>
+      <c r="D21" s="85" t="s">
+        <v>3984</v>
+      </c>
+      <c r="E21" s="85" t="s">
+        <v>3980</v>
+      </c>
+      <c r="G21" s="85" t="s">
+        <v>3929</v>
+      </c>
+      <c r="H21" s="85" t="s">
+        <v>3948</v>
+      </c>
+      <c r="I21" s="85" t="s">
+        <v>3949</v>
+      </c>
+      <c r="J21" s="85"/>
+      <c r="K21" s="85" t="s">
+        <v>3934</v>
+      </c>
+      <c r="L21" s="85" t="s">
+        <v>3971</v>
+      </c>
+      <c r="N21" s="85"/>
+    </row>
+    <row r="22" spans="2:14" ht="27" x14ac:dyDescent="0.35">
+      <c r="B22" s="85" t="s">
+        <v>1531</v>
+      </c>
+      <c r="C22" s="92">
+        <v>30</v>
+      </c>
+      <c r="D22" s="92">
+        <v>0.95</v>
+      </c>
+      <c r="E22" s="92">
+        <v>36085</v>
+      </c>
+      <c r="F22" s="92"/>
+      <c r="G22" s="47" t="s">
+        <v>3902</v>
+      </c>
+      <c r="H22" s="47">
+        <v>126.065</v>
+      </c>
+      <c r="I22" s="101">
+        <v>20.8201</v>
+      </c>
+      <c r="J22" s="93"/>
+      <c r="K22" s="93" t="s">
+        <v>3902</v>
+      </c>
+      <c r="L22" s="93">
+        <v>396.8</v>
+      </c>
+      <c r="N22" s="99"/>
+    </row>
+    <row r="23" spans="2:14" ht="27" x14ac:dyDescent="0.35">
+      <c r="B23" s="85" t="s">
+        <v>3979</v>
+      </c>
+      <c r="C23" s="92">
+        <v>23</v>
+      </c>
+      <c r="D23" s="92">
+        <v>0.9</v>
+      </c>
+      <c r="E23" s="92">
+        <v>16009</v>
+      </c>
+      <c r="F23" s="92"/>
+      <c r="G23" s="47" t="s">
+        <v>3902</v>
+      </c>
+      <c r="H23" s="47">
+        <v>390.51600000000002</v>
+      </c>
+      <c r="I23" s="101">
+        <v>275.56599999999997</v>
+      </c>
+      <c r="J23" s="93"/>
+      <c r="K23" s="93" t="s">
+        <v>3902</v>
+      </c>
+      <c r="L23" s="93" t="s">
+        <v>3902</v>
+      </c>
+      <c r="N23" s="99"/>
+    </row>
+    <row r="24" spans="2:14" ht="27" x14ac:dyDescent="0.35">
+      <c r="B24" s="85" t="s">
+        <v>1514</v>
+      </c>
+      <c r="C24" s="92">
+        <v>5</v>
+      </c>
+      <c r="D24" s="92">
+        <v>0.8</v>
+      </c>
+      <c r="E24" s="92">
+        <v>94500</v>
+      </c>
+      <c r="F24" s="92"/>
+      <c r="G24" s="47">
+        <v>50.255800000000001</v>
+      </c>
+      <c r="H24" s="47">
+        <v>50.8005</v>
+      </c>
+      <c r="I24" s="101">
+        <v>8.9690399999999997</v>
+      </c>
+      <c r="J24" s="93"/>
+      <c r="K24" s="93">
+        <v>235.078</v>
+      </c>
+      <c r="L24" s="93">
+        <v>296.74</v>
+      </c>
+      <c r="N24" s="99"/>
+    </row>
+    <row r="25" spans="2:14" ht="27" x14ac:dyDescent="0.35">
+      <c r="B25" s="85" t="s">
+        <v>1528</v>
+      </c>
+      <c r="C25" s="92">
+        <v>20</v>
+      </c>
+      <c r="D25" s="92">
+        <v>0.8</v>
+      </c>
+      <c r="E25" s="81">
+        <v>3785</v>
+      </c>
+      <c r="F25" s="92"/>
+      <c r="G25" s="47">
+        <v>1264.97</v>
+      </c>
+      <c r="H25" s="47">
+        <v>30.9161</v>
+      </c>
+      <c r="I25" s="101">
+        <v>30.710999999999999</v>
+      </c>
+      <c r="J25" s="93"/>
+      <c r="K25" s="93" t="s">
+        <v>3902</v>
+      </c>
+      <c r="L25" s="93" t="s">
+        <v>3902</v>
+      </c>
+      <c r="N25" s="99"/>
+    </row>
+    <row r="26" spans="2:14" ht="23" x14ac:dyDescent="0.3">
+      <c r="B26" s="81"/>
+      <c r="C26" s="92"/>
+      <c r="D26" s="92"/>
+      <c r="I26" s="94"/>
+      <c r="J26" s="94"/>
+    </row>
+    <row r="27" spans="2:14" ht="27" x14ac:dyDescent="0.35">
+      <c r="B27" s="100"/>
+      <c r="C27" s="92"/>
+      <c r="D27" s="92"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="O7:Q7"/>
     <mergeCell ref="S7:T7"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="K20:L20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
auto commit 2026-05-14 00:41:35
</commit_message>
<xml_diff>
--- a/results_BK_SM.xlsx
+++ b/results_BK_SM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/akahmad/Documents/G-ThinkerCG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A26C16B-92FC-A947-9E35-2C158E3C4CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15306CD-8394-D84F-B218-2FC924CDFCC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="6" xr2:uid="{93E1CCD5-64A0-5F4C-A5F1-EE4B217F183B}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6611" uniqueCount="3988">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6618" uniqueCount="3990">
   <si>
     <t>amazon0601</t>
   </si>
@@ -11928,6 +11928,9 @@
     <t>g2aimd</t>
   </si>
   <si>
+    <t>Trec</t>
+  </si>
+  <si>
     <t>Column7</t>
   </si>
   <si>
@@ -12010,6 +12013,9 @@
   </si>
   <si>
     <t>Time</t>
+  </si>
+  <si>
+    <t>fastqc final output</t>
   </si>
 </sst>
 </file>
@@ -12021,7 +12027,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="40" x14ac:knownFonts="1">
+  <fonts count="43" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -12161,6 +12167,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="18"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="14"/>
       <color theme="0" tint="-0.249977111117893"/>
       <name val="Aptos Narrow"/>
@@ -12244,28 +12256,41 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="14"/>
+      <sz val="18"/>
+      <name val="Monaco"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <name val="Monaco"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Monaco"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Monaco"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="14"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Aptos Display"/>
       <scheme val="major"/>
     </font>
     <font>
+      <b/>
       <sz val="18"/>
-      <name val="Monaco"/>
-      <family val="2"/>
+      <color theme="1"/>
+      <name val="Aptos Display"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="7">
@@ -12404,7 +12429,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -12445,8 +12470,8 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -12475,26 +12500,26 @@
     <xf numFmtId="2" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="24" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="24" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="24" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="25" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="25" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="25" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="24" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="25" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="25" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="20" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="26" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -12522,45 +12547,50 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="42" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -14583,10 +14613,10 @@
         <v>3932</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>3962</v>
+        <v>3963</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>3963</v>
+        <v>3964</v>
       </c>
       <c r="J5" s="13" t="s">
         <v>22</v>
@@ -14598,10 +14628,10 @@
         <v>24</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>3960</v>
+        <v>3961</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>3961</v>
+        <v>3962</v>
       </c>
       <c r="O5" s="12" t="s">
         <v>21</v>
@@ -14857,7 +14887,7 @@
         <v>215</v>
       </c>
       <c r="I16" s="89">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J16" s="41"/>
       <c r="K16" s="76"/>
@@ -27156,16 +27186,16 @@
         <v>3932</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>3975</v>
+        <v>3976</v>
       </c>
       <c r="I5" s="13" t="s">
         <v>20</v>
       </c>
       <c r="J5" s="13" t="s">
+        <v>3978</v>
+      </c>
+      <c r="K5" s="13" t="s">
         <v>3977</v>
-      </c>
-      <c r="K5" s="13" t="s">
-        <v>3976</v>
       </c>
       <c r="L5" s="13" t="s">
         <v>3929</v>
@@ -40619,7 +40649,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ED88F32-C306-9942-B2BF-61C867C9C8AC}">
-  <dimension ref="B4:AJ27"/>
+  <dimension ref="B3:AJ28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
@@ -40642,113 +40672,146 @@
     <col min="20" max="20" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="23.83203125" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:36" ht="19" x14ac:dyDescent="0.25">
-      <c r="W4" s="102" t="s">
-        <v>3972</v>
-      </c>
-      <c r="X4" s="102" t="s">
+    <row r="3" spans="2:36" x14ac:dyDescent="0.2">
+      <c r="N3" t="s">
+        <v>3989</v>
+      </c>
+    </row>
+    <row r="4" spans="2:36" ht="26" x14ac:dyDescent="0.35">
+      <c r="J4" t="s">
+        <v>3912</v>
+      </c>
+      <c r="K4">
+        <v>0.92</v>
+      </c>
+      <c r="L4">
+        <v>215</v>
+      </c>
+      <c r="N4">
+        <v>448192</v>
+      </c>
+      <c r="W4" s="106" t="s">
+        <v>3973</v>
+      </c>
+      <c r="X4" s="106" t="s">
+        <v>3986</v>
+      </c>
+      <c r="Y4" s="107"/>
+      <c r="Z4" s="107"/>
+      <c r="AA4" s="108" t="s">
+        <v>3942</v>
+      </c>
+      <c r="AB4" s="109" t="s">
+        <v>3988</v>
+      </c>
+      <c r="AC4" s="107"/>
+      <c r="AD4" s="108" t="s">
+        <v>3938</v>
+      </c>
+      <c r="AE4" s="109" t="s">
+        <v>3988</v>
+      </c>
+    </row>
+    <row r="5" spans="2:36" ht="26" x14ac:dyDescent="0.35">
+      <c r="J5" t="s">
+        <v>3960</v>
+      </c>
+      <c r="W5" s="106" t="s">
+        <v>3984</v>
+      </c>
+      <c r="X5" s="106">
+        <v>30</v>
+      </c>
+      <c r="Y5" s="107"/>
+      <c r="Z5" s="107"/>
+      <c r="AA5" s="110">
+        <v>100</v>
+      </c>
+      <c r="AB5" s="103">
+        <v>111.26600000000001</v>
+      </c>
+      <c r="AC5" s="107"/>
+      <c r="AD5" s="110">
+        <v>1</v>
+      </c>
+      <c r="AE5" s="102">
+        <v>19.003499999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="2:36" ht="26" x14ac:dyDescent="0.35">
+      <c r="W6" s="106" t="s">
         <v>3985</v>
       </c>
-      <c r="AA4" s="103" t="s">
-        <v>3942</v>
-      </c>
-      <c r="AB4" s="105" t="s">
-        <v>3987</v>
-      </c>
-      <c r="AD4" s="103" t="s">
-        <v>3938</v>
-      </c>
-      <c r="AE4" s="105" t="s">
-        <v>3987</v>
-      </c>
-    </row>
-    <row r="5" spans="2:36" ht="26" x14ac:dyDescent="0.35">
-      <c r="W5" s="102" t="s">
-        <v>3983</v>
-      </c>
-      <c r="X5" s="102">
-        <v>30</v>
-      </c>
-      <c r="AA5" s="104">
-        <v>100</v>
-      </c>
-      <c r="AB5" s="107">
-        <v>111.26600000000001</v>
-      </c>
-      <c r="AD5" s="104">
-        <v>1</v>
-      </c>
-      <c r="AE5" s="106">
-        <v>19.003499999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="2:36" ht="26" x14ac:dyDescent="0.35">
-      <c r="W6" s="102" t="s">
-        <v>3984</v>
-      </c>
-      <c r="X6" s="102">
+      <c r="X6" s="106">
         <v>0.95</v>
       </c>
-      <c r="AA6" s="104">
+      <c r="Y6" s="107"/>
+      <c r="Z6" s="107"/>
+      <c r="AA6" s="110">
         <v>1000</v>
       </c>
-      <c r="AB6" s="107">
+      <c r="AB6" s="103">
         <v>29.1617</v>
       </c>
-      <c r="AD6" s="104">
+      <c r="AC6" s="107"/>
+      <c r="AD6" s="110">
         <v>10</v>
       </c>
-      <c r="AE6" s="106">
+      <c r="AE6" s="102">
         <v>18.909700000000001</v>
       </c>
       <c r="AF6" s="90"/>
       <c r="AJ6" s="35"/>
     </row>
     <row r="7" spans="2:36" ht="27" x14ac:dyDescent="0.35">
-      <c r="O7" s="97"/>
-      <c r="P7" s="97"/>
-      <c r="Q7" s="97"/>
-      <c r="R7" s="96"/>
-      <c r="S7" s="95"/>
-      <c r="T7" s="95"/>
-      <c r="W7" s="102" t="s">
-        <v>3986</v>
-      </c>
-      <c r="X7" s="92">
+      <c r="O7" s="98"/>
+      <c r="P7" s="98"/>
+      <c r="Q7" s="98"/>
+      <c r="R7" s="97"/>
+      <c r="S7" s="96"/>
+      <c r="T7" s="96"/>
+      <c r="W7" s="106" t="s">
+        <v>3987</v>
+      </c>
+      <c r="X7" s="102">
         <v>36085</v>
       </c>
-      <c r="AA7" s="104">
+      <c r="Y7" s="107"/>
+      <c r="Z7" s="107"/>
+      <c r="AA7" s="111">
         <v>10000</v>
       </c>
-      <c r="AB7" s="107">
+      <c r="AB7" s="104">
         <v>18.9161</v>
       </c>
-      <c r="AD7" s="104">
+      <c r="AC7" s="107"/>
+      <c r="AD7" s="110">
         <v>20</v>
       </c>
-      <c r="AE7" s="106">
+      <c r="AE7" s="102">
         <v>17.566099999999999</v>
       </c>
       <c r="AF7" s="90"/>
     </row>
     <row r="8" spans="2:36" ht="27" x14ac:dyDescent="0.35">
       <c r="B8" s="85" t="s">
-        <v>3972</v>
+        <v>3973</v>
       </c>
       <c r="C8" s="85" t="s">
-        <v>3970</v>
+        <v>3971</v>
       </c>
       <c r="D8" s="85"/>
       <c r="E8" s="85" t="s">
-        <v>3973</v>
+        <v>3974</v>
       </c>
       <c r="F8" s="85" t="s">
         <v>3934</v>
       </c>
       <c r="G8" s="85" t="s">
-        <v>3971</v>
+        <v>3972</v>
       </c>
       <c r="J8" s="85"/>
       <c r="K8" s="85"/>
@@ -40760,23 +40823,28 @@
       <c r="R8" s="85"/>
       <c r="S8" s="85"/>
       <c r="T8" s="85"/>
-      <c r="AA8" s="104">
+      <c r="W8" s="107"/>
+      <c r="X8" s="107"/>
+      <c r="Y8" s="107"/>
+      <c r="Z8" s="107"/>
+      <c r="AA8" s="110">
         <v>20000</v>
       </c>
-      <c r="AB8" s="107">
+      <c r="AB8" s="103">
         <v>28.322800000000001</v>
       </c>
-      <c r="AD8" s="104">
+      <c r="AC8" s="107"/>
+      <c r="AD8" s="110">
         <v>50</v>
       </c>
-      <c r="AE8" s="106">
+      <c r="AE8" s="102">
         <v>20.896999999999998</v>
       </c>
       <c r="AF8" s="90"/>
     </row>
     <row r="9" spans="2:36" ht="27" x14ac:dyDescent="0.35">
       <c r="B9" s="83" t="s">
-        <v>3964</v>
+        <v>3965</v>
       </c>
       <c r="C9" s="88">
         <v>360</v>
@@ -40792,22 +40860,30 @@
         <v>0.01</v>
       </c>
       <c r="J9" s="85"/>
-      <c r="K9" s="92"/>
-      <c r="L9" s="92"/>
-      <c r="M9" s="92"/>
-      <c r="N9" s="92"/>
-      <c r="O9" s="93"/>
-      <c r="P9" s="93"/>
-      <c r="Q9" s="98"/>
-      <c r="R9" s="93"/>
-      <c r="S9" s="93"/>
-      <c r="T9" s="93"/>
-      <c r="AE9" s="91"/>
+      <c r="K9" s="93"/>
+      <c r="L9" s="93"/>
+      <c r="M9" s="93"/>
+      <c r="N9" s="93"/>
+      <c r="O9" s="94"/>
+      <c r="P9" s="94"/>
+      <c r="Q9" s="99"/>
+      <c r="R9" s="94"/>
+      <c r="S9" s="94"/>
+      <c r="T9" s="94"/>
+      <c r="W9" s="107"/>
+      <c r="X9" s="107"/>
+      <c r="Y9" s="107"/>
+      <c r="Z9" s="107"/>
+      <c r="AA9" s="107"/>
+      <c r="AB9" s="107"/>
+      <c r="AC9" s="107"/>
+      <c r="AD9" s="107"/>
+      <c r="AE9" s="112"/>
       <c r="AF9" s="90"/>
     </row>
     <row r="10" spans="2:36" ht="27" x14ac:dyDescent="0.35">
       <c r="B10" s="83" t="s">
-        <v>3965</v>
+        <v>3966</v>
       </c>
       <c r="C10" s="88">
         <v>6145</v>
@@ -40823,22 +40899,30 @@
         <v>0.22</v>
       </c>
       <c r="J10" s="85"/>
-      <c r="K10" s="92"/>
-      <c r="L10" s="92"/>
-      <c r="M10" s="92"/>
-      <c r="N10" s="92"/>
-      <c r="O10" s="93"/>
-      <c r="P10" s="93"/>
-      <c r="Q10" s="98"/>
-      <c r="R10" s="93"/>
-      <c r="S10" s="93"/>
-      <c r="T10" s="93"/>
-      <c r="AE10" s="91"/>
-      <c r="AF10" s="91"/>
+      <c r="K10" s="93"/>
+      <c r="L10" s="93"/>
+      <c r="M10" s="93"/>
+      <c r="N10" s="93"/>
+      <c r="O10" s="94"/>
+      <c r="P10" s="94"/>
+      <c r="Q10" s="99"/>
+      <c r="R10" s="94"/>
+      <c r="S10" s="94"/>
+      <c r="T10" s="94"/>
+      <c r="W10" s="107"/>
+      <c r="X10" s="107"/>
+      <c r="Y10" s="107"/>
+      <c r="Z10" s="107"/>
+      <c r="AA10" s="107"/>
+      <c r="AB10" s="107"/>
+      <c r="AC10" s="107"/>
+      <c r="AD10" s="107"/>
+      <c r="AE10" s="112"/>
+      <c r="AF10" s="92"/>
     </row>
     <row r="11" spans="2:36" ht="27" x14ac:dyDescent="0.35">
       <c r="B11" s="83" t="s">
-        <v>3966</v>
+        <v>3967</v>
       </c>
       <c r="C11" s="88">
         <v>28717</v>
@@ -40854,38 +40938,41 @@
         <v>49.23</v>
       </c>
       <c r="J11" s="85"/>
-      <c r="K11" s="92"/>
-      <c r="L11" s="92"/>
-      <c r="M11" s="92"/>
-      <c r="N11" s="92"/>
-      <c r="O11" s="93"/>
-      <c r="P11" s="93"/>
-      <c r="Q11" s="98"/>
-      <c r="R11" s="93"/>
-      <c r="S11" s="93"/>
-      <c r="T11" s="93"/>
-      <c r="W11" s="102" t="s">
-        <v>3972</v>
-      </c>
-      <c r="X11" s="102" t="s">
+      <c r="K11" s="93"/>
+      <c r="L11" s="93"/>
+      <c r="M11" s="93"/>
+      <c r="N11" s="93"/>
+      <c r="O11" s="94"/>
+      <c r="P11" s="94"/>
+      <c r="Q11" s="99"/>
+      <c r="R11" s="94"/>
+      <c r="S11" s="94"/>
+      <c r="T11" s="94"/>
+      <c r="W11" s="106" t="s">
+        <v>3973</v>
+      </c>
+      <c r="X11" s="106" t="s">
         <v>1528</v>
       </c>
-      <c r="AA11" s="103" t="s">
+      <c r="Y11" s="107"/>
+      <c r="Z11" s="107"/>
+      <c r="AA11" s="108" t="s">
         <v>3942</v>
       </c>
-      <c r="AB11" s="105" t="s">
-        <v>3987</v>
-      </c>
-      <c r="AD11" s="103" t="s">
+      <c r="AB11" s="109" t="s">
+        <v>3988</v>
+      </c>
+      <c r="AC11" s="107"/>
+      <c r="AD11" s="108" t="s">
         <v>3938</v>
       </c>
-      <c r="AE11" s="105" t="s">
-        <v>3987</v>
+      <c r="AE11" s="109" t="s">
+        <v>3988</v>
       </c>
     </row>
     <row r="12" spans="2:36" ht="27" x14ac:dyDescent="0.35">
       <c r="B12" s="83" t="s">
-        <v>3967</v>
+        <v>3968</v>
       </c>
       <c r="C12" s="88">
         <v>2517</v>
@@ -40901,38 +40988,41 @@
         <v>0.49</v>
       </c>
       <c r="J12" s="85"/>
-      <c r="K12" s="92"/>
-      <c r="L12" s="92"/>
-      <c r="M12" s="92"/>
-      <c r="N12" s="92"/>
-      <c r="O12" s="93"/>
-      <c r="P12" s="93"/>
-      <c r="Q12" s="93"/>
-      <c r="R12" s="93"/>
-      <c r="S12" s="93"/>
-      <c r="T12" s="98"/>
-      <c r="W12" s="102" t="s">
-        <v>3983</v>
-      </c>
-      <c r="X12" s="102">
+      <c r="K12" s="93"/>
+      <c r="L12" s="93"/>
+      <c r="M12" s="93"/>
+      <c r="N12" s="93"/>
+      <c r="O12" s="94"/>
+      <c r="P12" s="94"/>
+      <c r="Q12" s="94"/>
+      <c r="R12" s="94"/>
+      <c r="S12" s="94"/>
+      <c r="T12" s="99"/>
+      <c r="W12" s="106" t="s">
+        <v>3984</v>
+      </c>
+      <c r="X12" s="106">
         <v>20</v>
       </c>
-      <c r="AA12">
+      <c r="Y12" s="107"/>
+      <c r="Z12" s="107"/>
+      <c r="AA12" s="107">
         <v>10</v>
       </c>
-      <c r="AB12" s="82">
+      <c r="AB12" s="103">
         <v>112.94799999999999</v>
       </c>
-      <c r="AD12" s="104">
+      <c r="AC12" s="107"/>
+      <c r="AD12" s="110">
         <v>1</v>
       </c>
-      <c r="AE12" s="82">
+      <c r="AE12" s="103">
         <v>23.771899999999999</v>
       </c>
     </row>
-    <row r="13" spans="2:36" ht="23" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:36" ht="26" x14ac:dyDescent="0.35">
       <c r="B13" s="83" t="s">
-        <v>3968</v>
+        <v>3969</v>
       </c>
       <c r="C13" s="88">
         <v>24383</v>
@@ -40947,28 +41037,31 @@
       <c r="G13" s="87">
         <v>3.05</v>
       </c>
-      <c r="W13" s="102" t="s">
-        <v>3984</v>
-      </c>
-      <c r="X13" s="102">
+      <c r="W13" s="106" t="s">
+        <v>3985</v>
+      </c>
+      <c r="X13" s="106">
         <v>0.8</v>
       </c>
-      <c r="AA13" s="104">
+      <c r="Y13" s="107"/>
+      <c r="Z13" s="107"/>
+      <c r="AA13" s="110">
         <v>100</v>
       </c>
-      <c r="AB13" s="82">
+      <c r="AB13" s="103">
         <v>34.610700000000001</v>
       </c>
-      <c r="AD13" s="104">
+      <c r="AC13" s="107"/>
+      <c r="AD13" s="110">
         <v>10</v>
       </c>
-      <c r="AE13" s="82">
+      <c r="AE13" s="103">
         <v>23.1478</v>
       </c>
     </row>
-    <row r="14" spans="2:36" ht="23" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:36" ht="26" x14ac:dyDescent="0.35">
       <c r="B14" s="83" t="s">
-        <v>3969</v>
+        <v>3970</v>
       </c>
       <c r="C14" s="88">
         <v>8949</v>
@@ -40983,70 +41076,78 @@
       <c r="G14" s="87">
         <v>0.47</v>
       </c>
-      <c r="Q14" s="94"/>
-      <c r="R14" s="94"/>
-      <c r="W14" s="102" t="s">
-        <v>3986</v>
-      </c>
-      <c r="X14" s="92">
+      <c r="Q14" s="95"/>
+      <c r="R14" s="95"/>
+      <c r="W14" s="106" t="s">
+        <v>3987</v>
+      </c>
+      <c r="X14" s="102">
         <v>3785</v>
       </c>
-      <c r="AA14" s="104">
+      <c r="Y14" s="107"/>
+      <c r="Z14" s="107"/>
+      <c r="AA14" s="111">
         <v>1000</v>
       </c>
-      <c r="AB14" s="82">
+      <c r="AB14" s="104">
         <v>24.2639</v>
       </c>
-      <c r="AD14" s="104">
+      <c r="AC14" s="107"/>
+      <c r="AD14" s="110">
         <v>20</v>
       </c>
-      <c r="AE14" s="82">
+      <c r="AE14" s="103">
         <v>23.116099999999999</v>
       </c>
     </row>
-    <row r="15" spans="2:36" ht="22" x14ac:dyDescent="0.25">
-      <c r="AA15" s="104">
+    <row r="15" spans="2:36" ht="26" x14ac:dyDescent="0.35">
+      <c r="W15" s="107"/>
+      <c r="X15" s="107"/>
+      <c r="Y15" s="107"/>
+      <c r="Z15" s="107"/>
+      <c r="AA15" s="110">
         <v>10000</v>
       </c>
-      <c r="AB15" s="82">
+      <c r="AB15" s="103">
         <v>30.773599999999998</v>
       </c>
-      <c r="AD15" s="104">
+      <c r="AC15" s="107"/>
+      <c r="AD15" s="110">
         <v>50</v>
       </c>
-      <c r="AE15" s="82">
+      <c r="AE15" s="103">
         <v>24.661000000000001</v>
       </c>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
       <c r="F18" t="s">
-        <v>3974</v>
+        <v>3975</v>
       </c>
     </row>
     <row r="20" spans="2:14" ht="27" x14ac:dyDescent="0.35">
-      <c r="G20" s="97" t="s">
-        <v>3981</v>
-      </c>
-      <c r="H20" s="97"/>
-      <c r="I20" s="97"/>
-      <c r="J20" s="96"/>
-      <c r="K20" s="95" t="s">
+      <c r="G20" s="98" t="s">
         <v>3982</v>
       </c>
-      <c r="L20" s="95"/>
+      <c r="H20" s="98"/>
+      <c r="I20" s="98"/>
+      <c r="J20" s="97"/>
+      <c r="K20" s="96" t="s">
+        <v>3983</v>
+      </c>
+      <c r="L20" s="96"/>
     </row>
     <row r="21" spans="2:14" ht="27" x14ac:dyDescent="0.35">
       <c r="B21" s="85" t="s">
-        <v>3972</v>
+        <v>3973</v>
       </c>
       <c r="C21" s="85" t="s">
-        <v>3983</v>
+        <v>3984</v>
       </c>
       <c r="D21" s="85" t="s">
-        <v>3984</v>
+        <v>3985</v>
       </c>
       <c r="E21" s="85" t="s">
-        <v>3980</v>
+        <v>3981</v>
       </c>
       <c r="G21" s="85" t="s">
         <v>3929</v>
@@ -41062,7 +41163,7 @@
         <v>3934</v>
       </c>
       <c r="L21" s="85" t="s">
-        <v>3971</v>
+        <v>3972</v>
       </c>
       <c r="N21" s="85"/>
     </row>
@@ -41070,16 +41171,16 @@
       <c r="B22" s="85" t="s">
         <v>1531</v>
       </c>
-      <c r="C22" s="92">
+      <c r="C22" s="93">
         <v>30</v>
       </c>
-      <c r="D22" s="92">
+      <c r="D22" s="93">
         <v>0.95</v>
       </c>
-      <c r="E22" s="92">
+      <c r="E22" s="93">
         <v>36085</v>
       </c>
-      <c r="F22" s="92"/>
+      <c r="F22" s="93"/>
       <c r="G22" s="47" t="s">
         <v>3902</v>
       </c>
@@ -41089,29 +41190,29 @@
       <c r="I22" s="101">
         <v>20.8201</v>
       </c>
-      <c r="J22" s="93"/>
-      <c r="K22" s="93" t="s">
+      <c r="J22" s="94"/>
+      <c r="K22" s="94" t="s">
         <v>3902</v>
       </c>
-      <c r="L22" s="93">
+      <c r="L22" s="94">
         <v>396.8</v>
       </c>
-      <c r="N22" s="99"/>
+      <c r="N22" s="100"/>
     </row>
     <row r="23" spans="2:14" ht="27" x14ac:dyDescent="0.35">
       <c r="B23" s="85" t="s">
-        <v>3979</v>
-      </c>
-      <c r="C23" s="92">
+        <v>3980</v>
+      </c>
+      <c r="C23" s="93">
         <v>23</v>
       </c>
-      <c r="D23" s="92">
+      <c r="D23" s="93">
         <v>0.9</v>
       </c>
-      <c r="E23" s="92">
+      <c r="E23" s="93">
         <v>16009</v>
       </c>
-      <c r="F23" s="92"/>
+      <c r="F23" s="93"/>
       <c r="G23" s="47" t="s">
         <v>3902</v>
       </c>
@@ -41121,29 +41222,29 @@
       <c r="I23" s="101">
         <v>275.56599999999997</v>
       </c>
-      <c r="J23" s="93"/>
-      <c r="K23" s="93" t="s">
+      <c r="J23" s="94"/>
+      <c r="K23" s="94" t="s">
         <v>3902</v>
       </c>
-      <c r="L23" s="93" t="s">
+      <c r="L23" s="94" t="s">
         <v>3902</v>
       </c>
-      <c r="N23" s="99"/>
+      <c r="N23" s="100"/>
     </row>
     <row r="24" spans="2:14" ht="27" x14ac:dyDescent="0.35">
       <c r="B24" s="85" t="s">
         <v>1514</v>
       </c>
-      <c r="C24" s="92">
+      <c r="C24" s="93">
         <v>5</v>
       </c>
-      <c r="D24" s="92">
+      <c r="D24" s="93">
         <v>0.8</v>
       </c>
-      <c r="E24" s="92">
+      <c r="E24" s="93">
         <v>94500</v>
       </c>
-      <c r="F24" s="92"/>
+      <c r="F24" s="93"/>
       <c r="G24" s="47">
         <v>50.255800000000001</v>
       </c>
@@ -41153,29 +41254,29 @@
       <c r="I24" s="101">
         <v>8.9690399999999997</v>
       </c>
-      <c r="J24" s="93"/>
-      <c r="K24" s="93">
+      <c r="J24" s="94"/>
+      <c r="K24" s="94">
         <v>235.078</v>
       </c>
-      <c r="L24" s="93">
+      <c r="L24" s="94">
         <v>296.74</v>
       </c>
-      <c r="N24" s="99"/>
+      <c r="N24" s="100"/>
     </row>
     <row r="25" spans="2:14" ht="27" x14ac:dyDescent="0.35">
       <c r="B25" s="85" t="s">
         <v>1528</v>
       </c>
-      <c r="C25" s="92">
+      <c r="C25" s="93">
         <v>20</v>
       </c>
-      <c r="D25" s="92">
+      <c r="D25" s="93">
         <v>0.8</v>
       </c>
       <c r="E25" s="81">
         <v>3785</v>
       </c>
-      <c r="F25" s="92"/>
+      <c r="F25" s="93"/>
       <c r="G25" s="47">
         <v>1264.97</v>
       </c>
@@ -41185,26 +41286,74 @@
       <c r="I25" s="101">
         <v>30.710999999999999</v>
       </c>
-      <c r="J25" s="93"/>
-      <c r="K25" s="93" t="s">
+      <c r="J25" s="94"/>
+      <c r="K25" s="94" t="s">
         <v>3902</v>
       </c>
-      <c r="L25" s="93" t="s">
+      <c r="L25" s="94" t="s">
         <v>3902</v>
       </c>
-      <c r="N25" s="99"/>
-    </row>
-    <row r="26" spans="2:14" ht="23" x14ac:dyDescent="0.3">
-      <c r="B26" s="81"/>
-      <c r="C26" s="92"/>
-      <c r="D26" s="92"/>
-      <c r="I26" s="94"/>
-      <c r="J26" s="94"/>
-    </row>
-    <row r="27" spans="2:14" ht="27" x14ac:dyDescent="0.35">
-      <c r="B27" s="100"/>
-      <c r="C27" s="92"/>
-      <c r="D27" s="92"/>
+      <c r="N25" s="100"/>
+    </row>
+    <row r="26" spans="2:14" ht="22" x14ac:dyDescent="0.25">
+      <c r="B26" s="6" t="s">
+        <v>3960</v>
+      </c>
+      <c r="C26" s="93">
+        <v>115</v>
+      </c>
+      <c r="D26" s="93">
+        <v>0.96</v>
+      </c>
+      <c r="G26" s="91" t="s">
+        <v>3902</v>
+      </c>
+      <c r="H26" s="82">
+        <v>1087.48</v>
+      </c>
+      <c r="I26" s="105">
+        <v>996.42</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" ht="22" x14ac:dyDescent="0.25">
+      <c r="B27" s="81" t="s">
+        <v>3919</v>
+      </c>
+      <c r="C27" s="93">
+        <v>20</v>
+      </c>
+      <c r="D27" s="93">
+        <v>0.95</v>
+      </c>
+      <c r="G27" s="82">
+        <v>1708.14</v>
+      </c>
+      <c r="H27" s="82">
+        <v>1452.82</v>
+      </c>
+      <c r="I27" s="105">
+        <v>639.14099999999996</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14" ht="22" x14ac:dyDescent="0.25">
+      <c r="B28" s="6" t="s">
+        <v>3920</v>
+      </c>
+      <c r="C28" s="93">
+        <v>20</v>
+      </c>
+      <c r="D28" s="93">
+        <v>0.9</v>
+      </c>
+      <c r="G28" s="82">
+        <v>362.80500000000001</v>
+      </c>
+      <c r="H28" s="82">
+        <v>546.51199999999994</v>
+      </c>
+      <c r="I28" s="105">
+        <v>204.886</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -41288,10 +41437,10 @@
       </c>
       <c r="L2" s="5"/>
       <c r="Q2" t="s">
+        <v>3980</v>
+      </c>
+      <c r="R2" t="s">
         <v>3979</v>
-      </c>
-      <c r="R2" t="s">
-        <v>3978</v>
       </c>
     </row>
     <row r="3" spans="3:18" ht="21" x14ac:dyDescent="0.25">

</xml_diff>